<commit_message>
Sync site: nav/home polish, typography, YouTube URLs, founder timeline
- Home: HomeProse blocks, truth card sizing, English list/colon splitting
- Founder story: Phase A labels inline with timeline range
- Canonical YouTube: spirit medicine & universal matrix playlists, channel URL
- Add youtubeUrls; update achievements CTAs, siteContent UM placeholders
- Various UI: navbar, record/universal-matrix pages, i18n, page copy import

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/docs/page-copy/04-视频目录-灵魂档案.xlsx
+++ b/docs/page-copy/04-视频目录-灵魂档案.xlsx
@@ -398,15 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G68"/>
-  <cols>
-    <col min="1" max="1" width="36.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
-    <col min="5" max="5" width="72.83203125" customWidth="1"/>
-    <col min="6" max="6" width="48.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -534,10 +525,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D6" t="str">
-        <v>Close Dossier</v>
+        <v>Close abstract</v>
       </c>
       <c r="E6" t="str">
-        <v>关闭卷宗</v>
+        <v>关闭摘要</v>
       </c>
       <c r="F6" t="str">
         <v/>
@@ -603,10 +594,10 @@
         <v>button / link</v>
       </c>
       <c r="D9" t="str">
-        <v>Open Dossier</v>
+        <v>Abstract</v>
       </c>
       <c r="E9" t="str">
-        <v>打开卷宗</v>
+        <v>内容摘要</v>
       </c>
       <c r="F9" t="str">
         <v/>
@@ -652,7 +643,7 @@
         <v>Woos Record of Soul</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>吴氏灵体档案（纪录片）</v>
       </c>
       <c r="F11" t="str">
         <v/>
@@ -672,10 +663,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D12" t="str">
-        <v>This Documentary Was Shot Earlier, Recording The Process Of Woos Father And Son Being Possessed By Spirits And Fighting. And The Scientific Summary Of Human Research On Supernatural Phenomena, Near-Death Experience And Reincarnation.</v>
+        <v xml:space="preserve">This Documentary Was Shot Earlier, Recording the Scientific Summary Of Human Research On Supernatural Phenomena, Near-Death Experience And Reincarnation and the Process Of Woos Father And Son Being attached By Spirits And Fighting. </v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>此纪录片拍摄较早，记录了人类关于超自然现象，濒死体验，轮回等内容的研究汇总以及吴氏父子与附体灵体斗争的历史</v>
       </c>
       <c r="F12" t="str">
         <v/>
@@ -698,7 +689,7 @@
         <v>When Woos record of Soul were filmed, Spirits were sometimes called ghost and sometimes soul, but in the spirit medicine filmed in 2025, ghosts were clearly called spirit(ghost).</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>吴氏灵体档案拍摄时，灵体（鬼魂）有时被称作”鬼“或者”灵魂“，但在2025年拍摄的吴氏灵魂医学中，灵体”鬼魂“的叫法被正式确立</v>
       </c>
       <c r="F13" t="str">
         <v/>
@@ -767,7 +758,7 @@
         <v>FILE 1-1-1</v>
       </c>
       <c r="E16" t="str">
-        <v/>
+        <v>1-1-1系列</v>
       </c>
       <c r="F16" t="str">
         <v/>
@@ -790,7 +781,7 @@
         <v>Introduction to Woos Record of Soul</v>
       </c>
       <c r="E17" t="str">
-        <v/>
+        <v>摘要性介绍吴氏灵体档案系列视频的内容</v>
       </c>
       <c r="F17" t="str">
         <v/>
@@ -810,10 +801,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D18" t="str">
-        <v>An overview of the entire documentary , its methodology, and its revolutionary premise.</v>
+        <v xml:space="preserve">An overview of the entire documentary </v>
       </c>
       <c r="E18" t="str">
-        <v/>
+        <v>关于整个吴氏灵体档案的摘要</v>
       </c>
       <c r="F18" t="str">
         <v/>
@@ -836,7 +827,7 @@
         <v>17mins</v>
       </c>
       <c r="E19" t="str">
-        <v/>
+        <v>总时长17分钟</v>
       </c>
       <c r="F19" t="str">
         <v/>
@@ -859,7 +850,7 @@
         <v>FILE 1-1-2</v>
       </c>
       <c r="E20" t="str">
-        <v/>
+        <v>1-1-2系列</v>
       </c>
       <c r="F20" t="str">
         <v/>
@@ -882,7 +873,7 @@
         <v>Scientifically prove the Existence of Souls through Epilepsy</v>
       </c>
       <c r="E21" t="str">
-        <v/>
+        <v>如何用仪器科学地证明鬼魂真实的存在</v>
       </c>
       <c r="F21" t="str">
         <v/>
@@ -902,10 +893,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D22" t="str">
-        <v>Demonstrating how electromagnetic, thermal, and quantum sensors can detect and record phenomena attributable to spirit presence.</v>
+        <v>Demonstrating how EEG experiments can be applied to prove the existence of spirits ghosts</v>
       </c>
       <c r="E22" t="str">
-        <v/>
+        <v>阐明如何设计脑电图实验以科学验证灵体的存在</v>
       </c>
       <c r="F22" t="str">
         <v/>
@@ -928,7 +919,7 @@
         <v>6mins</v>
       </c>
       <c r="E23" t="str">
-        <v/>
+        <v>总时长6分钟</v>
       </c>
       <c r="F23" t="str">
         <v/>
@@ -951,7 +942,7 @@
         <v>FILE 1-1-3</v>
       </c>
       <c r="E24" t="str">
-        <v/>
+        <v>1-1-3系列</v>
       </c>
       <c r="F24" t="str">
         <v/>
@@ -974,7 +965,7 @@
         <v>Authenticity Research of PSI</v>
       </c>
       <c r="E25" t="str">
-        <v/>
+        <v>超自然（PSI）现象研究的真实性</v>
       </c>
       <c r="F25" t="str">
         <v/>
@@ -994,10 +985,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D26" t="str">
-        <v>PSI phenomena — telepathy, psychokinesis, clairvoyance — are the foundational gateway to understanding spiritual forces. Yet their legitimacy has long been dismissed as pseudoscience. This episode reveals groundbreaking research from China’s 507 Institute (China’s equivalent to NASA) — proving that spirit-derived forces are real, measurable, and reproducible.</v>
+        <v>The mysterious PSI phenomenon is the basis for uncovering the secrets of the soul and spiritual forces. However, the authenticity of PSI has never been confirmed. This series will showcase the astonishing scientific research of the 507 Institute (China's NASA) to explore the authenticity of the mysterious forces from the spiritual world</v>
       </c>
       <c r="E26" t="str">
-        <v/>
+        <v>神秘的PSI现象是揭秘灵魂和灵界力量的基础，但是PSI 的真实性一直没有被证实，本系列将展示中国507研究所(中国NASA)令人震惊的科学研究，来自灵界的神秘力量的真实性</v>
       </c>
       <c r="F26" t="str">
         <v/>
@@ -1017,10 +1008,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D27" t="str">
-        <v>Unprecedented high-speed camera footage and irrefutable PSI experimental data never before shown to the public. The authenticity of these experiments — rigorously controlled, peer-reviewed, and non-fakeable — forms the core of this video.</v>
+        <v>The series will unveil precious video footage captured by high-speed cameras that you've never seen before, and absolutely unfalsifiable PSI experiment materials that will broaden your horizons. The authenticity of the experiments is the essence and core of this series.</v>
       </c>
       <c r="E27" t="str">
-        <v/>
+        <v>你从未见过的高速摄影机拍摄的珍贵影像资料，以及完全不可作假的PSI实验材料将大开你的眼界。实验真实性是本系列的精华和核心</v>
       </c>
       <c r="F27" t="str">
         <v/>
@@ -1043,7 +1034,7 @@
         <v>64mins</v>
       </c>
       <c r="E28" t="str">
-        <v/>
+        <v>总时长64分钟</v>
       </c>
       <c r="F28" t="str">
         <v/>
@@ -1066,7 +1057,7 @@
         <v>FILE 1-2-1</v>
       </c>
       <c r="E29" t="str">
-        <v/>
+        <v>1-2-1系列</v>
       </c>
       <c r="F29" t="str">
         <v/>
@@ -1089,7 +1080,7 @@
         <v>Origin, Destination after death of Souls &amp; Impact on human</v>
       </c>
       <c r="E30" t="str">
-        <v/>
+        <v>人类鬼魂的来源和死后的去向，以及对人类的影响</v>
       </c>
       <c r="F30" t="str">
         <v/>
@@ -1098,7 +1089,7 @@
         <v>siteContent.recordOfSoul</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" xml:space="preserve">
       <c r="A31" t="str">
         <v>recordOfSoul.timeline[3].abstract</v>
       </c>
@@ -1108,11 +1099,12 @@
       <c r="C31" t="str">
         <v>paragraph / other</v>
       </c>
-      <c r="D31" t="str">
-        <v>Where do human souls come from? Where do they go after death? Do they ascend to heaven, descend to hell, or reincarnate according to religious doctrines?This episode reveals a startling truth: The primary destination of ancestral human spirits is not another realm — but parasitic attachment to living human beings.</v>
+      <c r="D31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Where does the human soul come from? Where does it go after death? Does it follow different religious divisions, going to different worlds? This video will thoroughly decode:
+the primary destination of the souls of human ancestors worldwide is to parasitize living humans!</v>
       </c>
       <c r="E31" t="str">
-        <v/>
+        <v>人类的灵魂从哪来的？人死后，灵魂到哪里去？是按照不同宗教的划分，去到不同的世界吗？本期视频将充分解密：全球人类祖先鬼魂的最主要的去向，是在活人身上寄生.鬼魂寄生人体，这些附体现象就会导致人类各种精神疾病。尤其是分离性障碍</v>
       </c>
       <c r="F31" t="str">
         <v/>
@@ -1132,10 +1124,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D32" t="str">
-        <v>Drawing on 12 peer-reviewed studies from Western universities and ICD-11 Category 6B6 (Spirit Attachment Disorders), this series maps the global distribution of spirit attachment and demonstrates its direct link to dissociative disorders, identity fragmentation, and unexplained psychological symptoms.</v>
+        <v>When a soul parasitizes a human body, this parasitism can lead to various mental illnesses, particularly dissociative disorders. This video series cites 12 papers from Western universities and the characteristics of class 6B6 diseases in the World Health Organization’s disease classification ICD-11, providing a comprehensive demonstration of the destinations and global distribution of souls and their impact on humanity.</v>
       </c>
       <c r="E32" t="str">
-        <v/>
+        <v>引用西方大学12篇论文以及世界卫生组织疾病分类ICD-11中的6B6类疾病，充分展示了鬼魂的去向和全球分布图谱以及对人类的影响</v>
       </c>
       <c r="F32" t="str">
         <v/>
@@ -1158,7 +1150,7 @@
         <v>154mins</v>
       </c>
       <c r="E33" t="str">
-        <v/>
+        <v>总时长154分钟</v>
       </c>
       <c r="F33" t="str">
         <v/>
@@ -1181,7 +1173,7 @@
         <v>FILE 1-2-2</v>
       </c>
       <c r="E34" t="str">
-        <v/>
+        <v>1-2-2系列</v>
       </c>
       <c r="F34" t="str">
         <v/>
@@ -1204,7 +1196,7 @@
         <v>Material Foundation of soul: Spiritual World has Natural Internet Attribute</v>
       </c>
       <c r="E35" t="str">
-        <v/>
+        <v>灵魂存在的根本性物质基础：灵虚世界天然具备接受意识上传的互联网属性</v>
       </c>
       <c r="F35" t="str">
         <v/>
@@ -1224,10 +1216,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D36" t="str">
-        <v>Traditional materialism denies spirit(Ghost) existence by asserting that consciousness is merely an epiphenomenon of the brain — and thus ceases at death. But Chinese PSI research proves otherwise: The ethereal realm possesses an innate, internet-like architecture capable of transmitting conscious information in GIF-like formats via a “blog-style” addressing system.This proves: Consciousness and the soul can exist independently of the physical brain.</v>
+        <v>Traditional materialism denies the existence of the soul on the basis that human consciousness is a byproduct of the brain, and consciousness completely ceases with the death of the brain. As the soul, being a secondary life form of human consciousness, naturally cannot exist independently. Supernatural experiments in China have proven that the spiritual world inherently possesses internet-like properties, capable of transmitting gif format consciousness image information, with information transmission addressing in the style of blogging. This demonstrates that consciousness and the soul can exist independently of the physical brain.</v>
       </c>
       <c r="E36" t="str">
-        <v/>
+        <v>传统唯物主义否定灵魂存在的根据是：人的意识是大脑的附属产物 ，意识随着大脑的死亡而完全消亡。灵魂作为人类意识类型的二次生命体，自然是不能独立存在的。中国的超自然实验证明：灵虚世界具备天然的互联网属性，可以传输gif格式的意识图片信息，信息传输寻址方式为博客方式。 由此证明，意识和灵魂可以独立于肉体大脑存在</v>
       </c>
       <c r="F36" t="str">
         <v/>
@@ -1247,10 +1239,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D37" t="str">
-        <v>Four groundbreaking PSI papers by Professor Shao Laisheng of Fudan University and colleagues demonstrate that humans can transmit pure conscious information — without instruments — from Shanghai to Beijing, directly through mental intent.</v>
+        <v>Four PSI scientific research papers by Professor Shao Lai Sheng and others from Fudan University in China have genuinely shown that, without the aid of any instruments, humans can send pure consciousness information from Shanghai to Beijing.</v>
       </c>
       <c r="E37" t="str">
-        <v/>
+        <v>中国复旦大学邵来圣教授等人的4篇PSI科学研究论文，真实的显示了，不借助任何仪器，人类可以从上海向北京发送纯意识信息</v>
       </c>
       <c r="F37" t="str">
         <v/>
@@ -1270,10 +1262,10 @@
         <v>label</v>
       </c>
       <c r="D38" t="str">
-        <v>32mins</v>
+        <v>35mins</v>
       </c>
       <c r="E38" t="str">
-        <v/>
+        <v>总时长35分钟</v>
       </c>
       <c r="F38" t="str">
         <v/>
@@ -1296,7 +1288,7 @@
         <v>FILE 1-2-3</v>
       </c>
       <c r="E39" t="str">
-        <v/>
+        <v>1-2-3系列</v>
       </c>
       <c r="F39" t="str">
         <v/>
@@ -1319,7 +1311,7 @@
         <v>Scientific Proof of Soul Parasitism/Possession caused Mental / Psychosis Illnesses</v>
       </c>
       <c r="E40" t="str">
-        <v/>
+        <v>各类精神病在人类群体中大规模存在，它们就是由鬼魂附体引发的疾病</v>
       </c>
       <c r="F40" t="str">
         <v/>
@@ -1339,10 +1331,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D41" t="str">
-        <v>In this world, where is it easy to find a spirit(ghost)? In countless patients with dissociative disorder, schizophrenia, epilepsy, depression, somatization disorder and many other diseases. This series of videos will deeply discuss the etiology research and pain brought by spirit(ghost) to mental patients.</v>
+        <v>IWhere in the world can souls be easily found? They are found in countless patients with dissociative disorders, schizophrenia, epilepsy, depression, somatization disorders, and many other diseases. This video series will deeply discuss the etiological research and suffering that spirits bring to mental patients</v>
       </c>
       <c r="E41" t="str">
-        <v/>
+        <v>在这个世界上，哪里很容易找到鬼魂？就在无数的分离性障碍、精神分裂症、癫痫、抑郁症、躯体化障碍等很多疾病患者身上。本系列视频将深度讨论鬼魂给精神病患者带来的病因研究和痛苦</v>
       </c>
       <c r="F41" t="str">
         <v/>
@@ -1362,10 +1354,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D42" t="str">
-        <v>This series of videos shows the distribution of spiritual body in the world with 15 medical research papers from famous western universities and precious real video materials of spirit(ghost) possession. The statistics of psychiatry are often the distribution data of spirit(ghost).</v>
+        <v xml:space="preserve"> This video series uses 15 medical research papers from famous Western universities, as well as precious real video materials of spirit possession / soul parasitism, to show the distribution of parasitic souls among humans. Psychiatric statistical data often represent the distribution of souls</v>
       </c>
       <c r="E42" t="str">
-        <v/>
+        <v>本系列视频用15篇西方著名大学的医学研究论文，以及珍贵的鬼魂附体真实视频资料展示了鬼魂在人间的分布。精神医学的统计资料往往就是鬼魂的分布资料</v>
       </c>
       <c r="F42" t="str">
         <v/>
@@ -1388,7 +1380,7 @@
         <v>154mins</v>
       </c>
       <c r="E43" t="str">
-        <v/>
+        <v>总时长154分钟</v>
       </c>
       <c r="F43" t="str">
         <v/>
@@ -1411,7 +1403,7 @@
         <v>FILE 1-2-4</v>
       </c>
       <c r="E44" t="str">
-        <v/>
+        <v>1-2-4系列</v>
       </c>
       <c r="F44" t="str">
         <v/>
@@ -1434,7 +1426,7 @@
         <v>Deep Exploration of Soul-triggering Epilepsy’s Mechanism</v>
       </c>
       <c r="E45" t="str">
-        <v/>
+        <v>鬼魂引发癫痫发作机制的深度探索</v>
       </c>
       <c r="F45" t="str">
         <v/>
@@ -1454,10 +1446,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D46" t="str">
-        <v>The Woos own epilepsy is caused by spirit(ghost) possession — directly contradicting modern neurology’s claim that epilepsy arises solely from abnormal neural firing. This series reveals: spirit(ghost) are material entities capable of emitting electromagnetic charges. These charges induce epileptogenic foci in the human brain, triggering seizures.</v>
+        <v>The epilepsy of the Woo father and son was caused by soul parasitism. This conflicts with the etiological theory of epilepsy in modern medicine. This video will reveal that souls have material properties and can release charges. The charges released by the souls cause the epileptic foci and seizures in the human brain.</v>
       </c>
       <c r="E46" t="str">
-        <v/>
+        <v>吴氏父子的癫痫是由鬼魂附体引起的。这和现代医学中癫痫的病因理论是相冲突的。本视频将揭示，鬼魂是物质属性的，可以释放电荷。鬼魂释放的电荷在人类大脑中造成了癫痫的病灶和癫痫的发作</v>
       </c>
       <c r="F46" t="str">
         <v/>
@@ -1477,10 +1469,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D47" t="str">
-        <v>Supported by 15 peer-reviewed medical papers from global universities and the Wu family’s personal medical records, this series provides irrefutable evidence that spirit-induced illness operates through physical, material mechanisms — not metaphysical mysticism.</v>
+        <v>The personal experiences of the Woo father and son, along with 15 medical papers from renowned universities worldwide, provide ample evidence that the disease-causing characteristics of souls have material properties</v>
       </c>
       <c r="E47" t="str">
-        <v/>
+        <v>全球15篇著名大学的医学论文以及吴氏父子的亲身经历充分证明了，鬼魂致病的特点是唯物属性的</v>
       </c>
       <c r="F47" t="str">
         <v/>
@@ -1503,7 +1495,7 @@
         <v>76mins</v>
       </c>
       <c r="E48" t="str">
-        <v/>
+        <v>总时长76分钟</v>
       </c>
       <c r="F48" t="str">
         <v/>
@@ -1526,7 +1518,7 @@
         <v>FILE 1-2-5</v>
       </c>
       <c r="E49" t="str">
-        <v/>
+        <v>1-2-5系列</v>
       </c>
       <c r="F49" t="str">
         <v/>
@@ -1549,7 +1541,7 @@
         <v>The truth of NDE – sophisticated illusions orchestrated by parasitic souls</v>
       </c>
       <c r="E50" t="str">
-        <v/>
+        <v>濒死体验真相揭秘---濒死体验只是附体鬼魂玩的把戏、制造的幻境</v>
       </c>
       <c r="F50" t="str">
         <v/>
@@ -1569,10 +1561,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D51" t="str">
-        <v>Near-death experiences (NDEs) — tunnels of light, deceased relatives, out-of-body journeys — are widely cited as proof of an afterlife. But this series proves: NDEs are not glimpses of death — they are hallucinations generated by attached spirits(ghosts). Through five analytical dimensions — consistency with other possession phenomena, visual structure, cross-cultural variation, and post-NDE psychic sequelae — this series dismantles the myth of NDEs as evidence of an afterlife.</v>
+        <v>This video series, through five sections examining the consistency between near-death experiences and other soul possession phenomena, visual studies of near-death experiences, differences in near-death experiences among various countries and religious and cultural backgrounds, and supernatural sequelae after near-death experiences, proves that near-death experiences are not the truth about what happens after death.</v>
       </c>
       <c r="E51" t="str">
-        <v/>
+        <v>本系列视频从濒死体验与其他鬼魂附体现象的一致性、濒死体验的视觉研究、濒死体验在不同国家和宗教、文化之间的差异、濒死体验后的超自然后遗症等5个板块证明：濒死体验并非死后真相</v>
       </c>
       <c r="F51" t="str">
         <v/>
@@ -1592,10 +1584,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D52" t="str">
-        <v>A deep analysis of 34 peer-reviewed NDE studies from top Western universities. Unlike popular media, which cherry-pick romanticized accounts, this series presents the full, unfiltered dataset — revealing NDEs as culturally conditioned, neurobiologically induced illusions orchestrated by spirit entities.</v>
+        <v>Many movies and books describe near-death experiences, using them as evidence to prove the existence and destination of religion and the soul. However, these cultural works do not fully display all the data and true data of near-death experiences to the public. This video series deeply excavates 34 research papers on near-death experiences from famous Western universities, fully revealing the truth about near-death experiences.</v>
       </c>
       <c r="E52" t="str">
-        <v/>
+        <v>很多电影和书籍都在描述濒死体验，把濒死体验作为证明宗教和灵魂存在和去向的证据。但是这些文化作品没有把濒死体验全部的数据和真实的数据展示给大众。本系列视频深度挖掘了西方著名大学34篇濒死体验的研究论文，全方位揭示了濒死体验的真相</v>
       </c>
       <c r="F52" t="str">
         <v/>
@@ -1618,7 +1610,7 @@
         <v>74mins</v>
       </c>
       <c r="E53" t="str">
-        <v/>
+        <v>总时长74分钟</v>
       </c>
       <c r="F53" t="str">
         <v/>
@@ -1641,7 +1633,7 @@
         <v>FILE 1-2-6</v>
       </c>
       <c r="E54" t="str">
-        <v/>
+        <v>1-2-6系列</v>
       </c>
       <c r="F54" t="str">
         <v/>
@@ -1664,7 +1656,7 @@
         <v>Past life memories come from parasitic souls, it can not prove reincarnation</v>
       </c>
       <c r="E55" t="str">
-        <v/>
+        <v>前世记忆的真相---前世记忆只是附体鬼魂将自己的记忆输入给宿主，它不能证明轮回存在</v>
       </c>
       <c r="F55" t="str">
         <v/>
@@ -1684,10 +1676,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D56" t="str">
-        <v>Through the human mind’s “consciousness input port” — particularly the memory system — attached spirits(ghosts) transmit their own life experiences in first-person narrative form. The host misinterprets these as their own past-life memories, leading to the widespread belief in reincarnation. This series demonstrates that reincarnation is a cognitive illusion, not a metaphysical reality.</v>
+        <v>Through the consciousness port of the human body, especially the memory input port, the parasitic soul inputs its own life in the form of first-person memories to the host. The host mistakenly believes that this memory is the life of their past lives, thereby generating the concept of reincarnation. This is a major misunderstanding in the study of spirituality.</v>
       </c>
       <c r="E56" t="str">
-        <v/>
+        <v>通过人体的意识端口，特别是记忆输入端口，附体鬼魂将自己生活，以第1人称形式的记忆输入给宿主。宿主误以为此记忆是自己的前世生活，并由此产生了轮回的概念。是灵学研究很大的误区</v>
       </c>
       <c r="F56" t="str">
         <v/>
@@ -1707,10 +1699,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D57" t="str">
-        <v>Rigorous logical analysis: The alleged “reincarnated self” has no biological continuity. It lacks a coherent sense of “I” — no unified identity, no persistent consciousness. Memory transfer ≠ identity transfer. This series exposes a fundamental error in spiritual research: mistaking information transfer for soul migration.</v>
+        <v>Deep logical reasoning derived from the concept of reincarnation produced by past-life memories – the subject of reincarnation does not have life characteristics; the subject of reincarnation does not have the concept of " I "</v>
       </c>
       <c r="E57" t="str">
-        <v/>
+        <v>由前世记忆产生轮回概念的深度逻辑推理---轮回的主体没有生命特征；轮回的主体没有“我”的概念</v>
       </c>
       <c r="F57" t="str">
         <v/>
@@ -1733,7 +1725,7 @@
         <v>42mins</v>
       </c>
       <c r="E58" t="str">
-        <v/>
+        <v>总时长42分钟</v>
       </c>
       <c r="F58" t="str">
         <v/>
@@ -1756,7 +1748,7 @@
         <v>FILE 1-3</v>
       </c>
       <c r="E59" t="str">
-        <v/>
+        <v>1-3系列</v>
       </c>
       <c r="F59" t="str">
         <v/>
@@ -1779,7 +1771,7 @@
         <v>Whether Souls have Eyes? Scientific Discovery on Spiritual Vision</v>
       </c>
       <c r="E60" t="str">
-        <v/>
+        <v>灵体是否有眼睛</v>
       </c>
       <c r="F60" t="str">
         <v/>
@@ -1788,7 +1780,7 @@
         <v>siteContent.recordOfSoul</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" xml:space="preserve">
       <c r="A61" t="str">
         <v>recordOfSoul.timeline[9].abstract</v>
       </c>
@@ -1798,11 +1790,13 @@
       <c r="C61" t="str">
         <v>paragraph / other</v>
       </c>
-      <c r="D61" t="str">
-        <v>Eyes are a fundamental condition shaping the very nature of spirits(ghost) existence. If spirits(ghost) lack eyes, this fundamentally challenges every cultural, religious, and metaphysical assumption about the afterlife. Across nearly all human cultures, the ethereal realm is depicted as containing hellfires, paradisiacal realms, demons, gods, and other spirits. But how can spirits(ghost) perceive these environments — or each other — without visual organs? How can the imagined existence of spirits(ghost) even be coherent without sight?</v>
-      </c>
-      <c r="E61" t="str">
-        <v/>
+      <c r="D61" t="str" xml:space="preserve">
+        <v xml:space="preserve">Eyes are the fundamental condition that affects the living style of ghosts. Ghosts without eyes will subvert everyone's spiritual view.
+Most cultures in the world believe that there is hell in the spiritual world. If ghosts have no eyes, how can they see the flames of hell or the beautiful scenery of Elysium? How can ghosts see other ghosts, demons or immortals? How can you imagine the ghost's living state and living environment when watching the video?</v>
+      </c>
+      <c r="E61" t="str" xml:space="preserve">
+        <v xml:space="preserve">眼睛是影响鬼魂生存方式的根本条件。鬼魂没有眼睛，将颠覆每个人的灵学观
+全世界绝大多数文化都认为灵虚世界存在地狱，如果鬼魂没有眼睛，鬼魂如何看得见地狱的火焰或者极乐世界的美景？鬼魂如何看得见其他的鬼、恶魔或者神仙？看视频的你想象中的鬼魂生存状态和生存环境又怎能存在？</v>
       </c>
       <c r="F61" t="str">
         <v/>
@@ -1822,10 +1816,10 @@
         <v>paragraph / other</v>
       </c>
       <c r="D62" t="str">
-        <v>This series draws upon 19 peer-reviewed academic papers from China’s most prestigious institutions — including the Institute of Physics and Institute of Biophysics (Chinese Academy of Sciences), Peking University, National Taiwan University, Beijing Normal University, and the Shanghai Institute of Laser Technology — combined with the firsthand experiential accounts of the Wu family. Collectively, they provide conclusive evidence: spirits(ghost) do not possess eyes.</v>
+        <v>This series of videos quotes the Institute of Physics and the Institute of Biophysics, Chinese Academy of Sciences; 19 research papers written by professors and scholars from Peking University, National Taiwan University, Beijing Normal University, Shanghai Institute of Laser Technology and other units, as well as the personal experience of Woo's father and son, fully prove that souls Have no eyes</v>
       </c>
       <c r="E62" t="str">
-        <v/>
+        <v>本系列视频引用了中国科学院物理研究所、生物物理研究所；北京大学，台湾大学，北京师范学院，上海激光技术研究所等单位的教授和学者撰写的19篇研究论文以及吴氏父子的亲身经历，充分证明：鬼魂没有眼睛</v>
       </c>
       <c r="F62" t="str">
         <v/>
@@ -1848,7 +1842,7 @@
         <v>77mins</v>
       </c>
       <c r="E63" t="str">
-        <v/>
+        <v>总时长77分钟</v>
       </c>
       <c r="F63" t="str">
         <v/>
@@ -1871,7 +1865,7 @@
         <v>FILE 1-4</v>
       </c>
       <c r="E64" t="str">
-        <v/>
+        <v>1-4系列</v>
       </c>
       <c r="F64" t="str">
         <v/>
@@ -1894,7 +1888,7 @@
         <v>Discover the truth of body shape, organs, material composition and metabolism of souls</v>
       </c>
       <c r="E65" t="str">
-        <v/>
+        <v>全面解密鬼魂的身体形状和器官、身体物质构成及能量代谢体系</v>
       </c>
       <c r="F65" t="str">
         <v/>
@@ -1917,7 +1911,7 @@
         <v>The ethereal body is material in nature. This series represents the first systematic scientific exploration into the physical structure, organ systems, material composition, and energy metabolism of human spirits(soul) after death — marking humanity’s initial step toward understanding the material reality of the ethereal realm.</v>
       </c>
       <c r="E66" t="str">
-        <v/>
+        <v>鬼魂的身体是物质属性的，本系列将初步解密人类死后鬼魂的身体形状和器官、身体物质构成及能量代谢体系。也是人类向鬼魂和灵虚世界物质构成探索，迈出的第1步</v>
       </c>
       <c r="F66" t="str">
         <v/>
@@ -1940,7 +1934,7 @@
         <v>Drawing on 8 international academic studies, the ICD-11 classification (Category 6B6: Spirit Attachment Disorders) from the World Health Organization, and rare archival footage, this series presents the most comprehensive and empirically grounded analysis to date of the spirit body’s anatomical and physiological characteristics..</v>
       </c>
       <c r="E67" t="str">
-        <v/>
+        <v>本系列视频引用全球8篇各类型学术研究论文，世界卫生组织疾病分类ICD-11中6B6类疾病的特征，以及罕见的视频资料。大规模、充分阐述了鬼魂身体的各项特征</v>
       </c>
       <c r="F67" t="str">
         <v/>
@@ -1963,7 +1957,7 @@
         <v>243mins</v>
       </c>
       <c r="E68" t="str">
-        <v/>
+        <v>总时长243分钟</v>
       </c>
       <c r="F68" t="str">
         <v/>

</xml_diff>